<commit_message>
Added data exploration and data sources
</commit_message>
<xml_diff>
--- a/Sources.xlsx
+++ b/Sources.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\natal\OneDrive\Pulpit\DSBA - UW\Semestr 2\Econometrics\Final Paper\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\natal\OneDrive\Pulpit\DSBA - UW\Semestr 2\Econometrics\Final Paper\econometrics-project\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FFF6E581-A372-4B5A-A3D1-DBCFEEF19673}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2DA2E3A2-97B2-46C2-BC18-EA807A9326DE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{C38F9C38-71EE-4F16-8524-A9649EDB3FDC}"/>
   </bookViews>
@@ -37,9 +37,6 @@
   </si>
   <si>
     <t>Series code / notes</t>
-  </si>
-  <si>
-    <t>Unemployment benefits (% GDP)</t>
   </si>
   <si>
     <t>ILO ILOSTAT</t>
@@ -316,6 +313,9 @@
 kinship_df &lt;- country_data %&gt;%
   select(isocode, country, kinship_score)
 write.csv(kinship_df, "kinship_df.csv", row.names = FALSE)</t>
+  </si>
+  <si>
+    <t>Proportion of population covered by social protection</t>
   </si>
 </sst>
 </file>
@@ -759,126 +759,126 @@
         <v>3</v>
       </c>
       <c r="E1" s="8" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="F1" s="2" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="G1" s="2" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
     </row>
     <row r="2" spans="1:7" ht="216">
       <c r="A2" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="B2" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="B2" s="4" t="s">
+      <c r="C2" s="1" t="s">
         <v>5</v>
-      </c>
-      <c r="C2" s="1" t="s">
-        <v>6</v>
       </c>
       <c r="D2" s="4" t="s">
         <v>0</v>
       </c>
       <c r="E2" s="9" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="F2" s="1" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
     </row>
     <row r="3" spans="1:7" ht="133.80000000000001" customHeight="1">
       <c r="A3" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="B3" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="B3" s="4" t="s">
+      <c r="C3" s="5" t="s">
         <v>8</v>
       </c>
-      <c r="C3" s="5" t="s">
-        <v>9</v>
-      </c>
       <c r="D3" s="4" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="E3" s="9" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="F3" s="1" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
     </row>
     <row r="4" spans="1:7" ht="99" customHeight="1">
       <c r="A4" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="B4" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="C4" s="5" t="s">
         <v>10</v>
       </c>
-      <c r="B4" s="4" t="s">
-        <v>8</v>
-      </c>
-      <c r="C4" s="5" t="s">
-        <v>11</v>
-      </c>
       <c r="D4" s="4" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="E4" s="9" t="s">
+        <v>26</v>
+      </c>
+      <c r="F4" s="1" t="s">
         <v>27</v>
-      </c>
-      <c r="F4" s="1" t="s">
-        <v>28</v>
       </c>
     </row>
     <row r="5" spans="1:7" ht="139.19999999999999" customHeight="1">
       <c r="A5" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="B5" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="C5" s="5" t="s">
         <v>12</v>
       </c>
-      <c r="B5" s="4" t="s">
-        <v>8</v>
-      </c>
-      <c r="C5" s="5" t="s">
-        <v>13</v>
-      </c>
       <c r="D5" s="4" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="E5" s="9" t="s">
+        <v>28</v>
+      </c>
+      <c r="F5" s="1" t="s">
         <v>29</v>
-      </c>
-      <c r="F5" s="1" t="s">
-        <v>30</v>
       </c>
     </row>
     <row r="6" spans="1:7" ht="141" customHeight="1">
       <c r="A6" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="B6" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="B6" s="4" t="s">
+      <c r="C6" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="C6" s="1" t="s">
-        <v>16</v>
-      </c>
       <c r="D6" s="4" t="s">
+        <v>33</v>
+      </c>
+      <c r="E6" s="11" t="s">
+        <v>32</v>
+      </c>
+      <c r="F6" s="7" t="s">
         <v>34</v>
       </c>
-      <c r="E6" s="11" t="s">
-        <v>33</v>
-      </c>
-      <c r="F6" s="7" t="s">
-        <v>35</v>
-      </c>
       <c r="G6" s="1" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
     </row>
     <row r="7" spans="1:7" ht="331.2">
       <c r="A7" s="1" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B7" s="2"/>
       <c r="C7" s="1"/>
       <c r="F7" s="1" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
     </row>
   </sheetData>

</xml_diff>